<commit_message>
Align journeys and capabilities with the reference postpaid/prepaid journeys
Prepaid and postpaid Add-ons redesign, ChoiceCards, single Address layout, fixed-line plan cards in Plan Selection, MNP postpaid on the shared plan/checkout/CAF steps, Pre-to-Post rebuilt on shared steps, capability samples per variant, dead legacy wizard removed, workbooks regenerated.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vfq-dxp-app/reference/outputs/01 Test_Data.xlsx
+++ b/vfq-dxp-app/reference/outputs/01 Test_Data.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/parithimalsaravanan/claude-projects/vfq/vfq-dxp-app/reference/outputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CA87E13-7429-2541-9AA3-322A1A0345BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C9E0F50-CC2D-0144-9AB1-4F6F6646B59C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="34560" windowHeight="21000" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="23" r:id="rId1"/>
-    <sheet name="Persona by Approach" sheetId="3" r:id="rId2"/>
-    <sheet name="Login Credentials" sheetId="4" r:id="rId3"/>
+    <sheet name="Login Credentials" sheetId="4" r:id="rId1"/>
+    <sheet name="Login" sheetId="23" r:id="rId2"/>
+    <sheet name="Persona by Approach" sheetId="3" r:id="rId3"/>
     <sheet name="Scenarios" sheetId="22" r:id="rId4"/>
     <sheet name="Customer Search" sheetId="5" r:id="rId5"/>
     <sheet name="Global Search" sheetId="6" r:id="rId6"/>
@@ -40,15 +40,15 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Customer Search'!$A$1:$J$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'ID Lookup (MOI Fetch)'!$A$1:$G$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Login Credentials'!$A$1:$J$29</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Persona by Approach'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Login Credentials'!$A$1:$J$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Persona by Approach'!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1510" uniqueCount="915">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1537" uniqueCount="915">
   <si>
     <t>Staff ID</t>
   </si>
@@ -2992,7 +2992,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -3156,7 +3156,6 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -3479,478 +3478,959 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1908BFEF-047E-5F45-B558-E6F9CE558EF2}">
-  <dimension ref="A1:E27"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="18" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:J29"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.85546875" defaultRowHeight="18" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="13" customWidth="1"/>
-    <col min="3" max="3" width="44.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="44.5703125" customWidth="1"/>
-    <col min="5" max="5" width="39.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.5703125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="22.42578125" style="3" customWidth="1"/>
+    <col min="3" max="3" width="34.5703125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="29.7109375" style="3" customWidth="1"/>
+    <col min="5" max="5" width="27" style="3" customWidth="1"/>
+    <col min="6" max="6" width="24.28515625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="32.42578125" style="3" customWidth="1"/>
+    <col min="8" max="8" width="24.28515625" style="3" customWidth="1"/>
+    <col min="9" max="9" width="21.5703125" style="3" customWidth="1"/>
+    <col min="10" max="10" width="81" style="3" customWidth="1"/>
+    <col min="11" max="13" width="11.85546875" style="1" customWidth="1"/>
+    <col min="14" max="16384" width="11.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" s="57" t="s">
-        <v>881</v>
-      </c>
-      <c r="B1" s="57" t="s">
+    <row r="1" spans="1:10" ht="19" x14ac:dyDescent="0.2">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="57" t="s">
-        <v>630</v>
-      </c>
-      <c r="D1" s="57" t="s">
-        <v>914</v>
-      </c>
-      <c r="E1" s="57" t="s">
-        <v>882</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>883</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="B1" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="57" x14ac:dyDescent="0.2">
+      <c r="A2" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B2" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="E2" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>884</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="I2" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="15" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="38" x14ac:dyDescent="0.2">
+      <c r="A3" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="C3" t="s">
+      <c r="B3" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="G3" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E3" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>885</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="I3" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="J3" s="15" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="57" x14ac:dyDescent="0.2">
+      <c r="A4" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="C4" t="s">
+      <c r="B4" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="D4" t="s">
-        <v>250</v>
-      </c>
-      <c r="E4" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>886</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="D4" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="G4" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="H4" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="I4" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" s="15" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="38" x14ac:dyDescent="0.2">
+      <c r="A5" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="C5" t="s">
+      <c r="B5" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="F5" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="G5" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="H5" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="E5" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>887</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="I5" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="J5" s="15" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="38" x14ac:dyDescent="0.2">
+      <c r="A6" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="C6" t="s">
+      <c r="B6" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="G6" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="H6" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E6" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>888</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="I6" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="J6" s="15" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="57" x14ac:dyDescent="0.2">
+      <c r="A7" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="C7" t="s">
+      <c r="B7" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="G7" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="E7" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>889</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="H7" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="I7" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="J7" s="15" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="57" x14ac:dyDescent="0.2">
+      <c r="A8" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="C8" t="s">
+      <c r="B8" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="G8" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="E8" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>890</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="H8" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="I8" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="J8" s="15" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="38" x14ac:dyDescent="0.2">
+      <c r="A9" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="C9" t="s">
+      <c r="B9" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="G9" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="E9" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>891</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="H9" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="I9" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="J9" s="15" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="38" x14ac:dyDescent="0.2">
+      <c r="A10" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="C10" t="s">
+      <c r="B10" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="F10" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="G10" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="E10" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>892</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="H10" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="I10" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="J10" s="15" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="57" x14ac:dyDescent="0.2">
+      <c r="A11" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="C11" t="s">
+      <c r="B11" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="F11" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="G11" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="H11" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="E11" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>893</v>
-      </c>
-      <c r="B12" t="s">
+      <c r="I11" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="J11" s="15" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="57" x14ac:dyDescent="0.2">
+      <c r="A12" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="C12" t="s">
+      <c r="B12" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="E12" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="F12" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="G12" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="H12" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="E12" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>894</v>
-      </c>
-      <c r="B13" t="s">
+      <c r="I12" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="J12" s="15" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="57" x14ac:dyDescent="0.2">
+      <c r="A13" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="C13" t="s">
+      <c r="B13" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="D13" t="s">
-        <v>271</v>
-      </c>
-      <c r="E13" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>895</v>
-      </c>
-      <c r="B14" t="s">
+      <c r="D13" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="E13" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" s="15" t="s">
+        <v>93</v>
+      </c>
+      <c r="G13" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="H13" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="I13" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="J13" s="15" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="38" x14ac:dyDescent="0.2">
+      <c r="A14" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="C14" t="s">
+      <c r="B14" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" s="15" t="s">
         <v>98</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="E14" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="F14" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="G14" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="H14" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="E14" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>896</v>
-      </c>
-      <c r="B15" t="s">
+      <c r="I14" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="J14" s="15" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="57" x14ac:dyDescent="0.2">
+      <c r="A15" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="D15" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="E15" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="F15" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="G15" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="H15" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="I15" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="J15" s="15" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="57" x14ac:dyDescent="0.2">
+      <c r="A16" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C16" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="D16" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="E16" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="F16" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="G16" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="H16" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="I16" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="J16" s="15" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="57" x14ac:dyDescent="0.2">
+      <c r="A17" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="B17" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="D17" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="E17" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="F17" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="G17" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="H17" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="I17" s="15" t="s">
+        <v>121</v>
+      </c>
+      <c r="J17" s="15" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="38" x14ac:dyDescent="0.2">
+      <c r="A18" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="B18" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="D18" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="E18" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="F18" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="G18" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="H18" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="I18" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="J18" s="15" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="76" x14ac:dyDescent="0.2">
+      <c r="A19" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="D19" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="E19" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="F19" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="G19" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="H19" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="I19" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="J19" s="15" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="76" x14ac:dyDescent="0.2">
+      <c r="A20" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C20" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="D20" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="E20" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="F20" s="15" t="s">
+        <v>138</v>
+      </c>
+      <c r="G20" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="H20" s="15" t="s">
+        <v>139</v>
+      </c>
+      <c r="I20" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="J20" s="15" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="57" x14ac:dyDescent="0.2">
+      <c r="A21" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C21" s="15" t="s">
+        <v>142</v>
+      </c>
+      <c r="D21" s="15" t="s">
+        <v>143</v>
+      </c>
+      <c r="E21" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="F21" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="G21" s="15" t="s">
+        <v>142</v>
+      </c>
+      <c r="H21" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="I21" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="J21" s="15" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="38" x14ac:dyDescent="0.2">
+      <c r="A22" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C22" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="D22" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="E22" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="F22" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="G22" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="H22" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="I22" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="J22" s="15" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="57" x14ac:dyDescent="0.2">
+      <c r="A23" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="B23" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C23" s="15" t="s">
+        <v>156</v>
+      </c>
+      <c r="D23" s="15" t="s">
+        <v>157</v>
+      </c>
+      <c r="E23" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="F23" s="15" t="s">
+        <v>158</v>
+      </c>
+      <c r="G23" s="15" t="s">
+        <v>156</v>
+      </c>
+      <c r="H23" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="I23" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="J23" s="15" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="57" x14ac:dyDescent="0.2">
+      <c r="A24" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C24" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="D24" s="15" t="s">
+        <v>157</v>
+      </c>
+      <c r="E24" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="F24" s="15" t="s">
+        <v>164</v>
+      </c>
+      <c r="G24" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="H24" s="15" t="s">
+        <v>166</v>
+      </c>
+      <c r="I24" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="J24" s="15" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="57" x14ac:dyDescent="0.2">
+      <c r="A25" s="15" t="s">
+        <v>168</v>
+      </c>
+      <c r="B25" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C25" s="15" t="s">
+        <v>169</v>
+      </c>
+      <c r="D25" s="15" t="s">
+        <v>170</v>
+      </c>
+      <c r="E25" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="F25" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="G25" s="15" t="s">
+        <v>169</v>
+      </c>
+      <c r="H25" s="15" t="s">
+        <v>172</v>
+      </c>
+      <c r="I25" s="15" t="s">
+        <v>173</v>
+      </c>
+      <c r="J25" s="15" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="38" x14ac:dyDescent="0.2">
+      <c r="A26" s="15" t="s">
+        <v>175</v>
+      </c>
+      <c r="B26" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C26" s="15" t="s">
+        <v>176</v>
+      </c>
+      <c r="D26" s="15" t="s">
+        <v>177</v>
+      </c>
+      <c r="E26" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="F26" s="15" t="s">
+        <v>178</v>
+      </c>
+      <c r="G26" s="15" t="s">
+        <v>176</v>
+      </c>
+      <c r="H26" s="15" t="s">
+        <v>179</v>
+      </c>
+      <c r="I26" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="J26" s="15" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="76" x14ac:dyDescent="0.2">
+      <c r="A27" s="15" t="s">
         <v>182</v>
       </c>
-      <c r="C15" t="s">
+      <c r="B27" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C27" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="D15" t="s">
-        <v>909</v>
-      </c>
-      <c r="E15" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>897</v>
-      </c>
-      <c r="B16" t="s">
-        <v>104</v>
-      </c>
-      <c r="C16" t="s">
-        <v>105</v>
-      </c>
-      <c r="D16" t="s">
-        <v>910</v>
-      </c>
-      <c r="E16" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>898</v>
-      </c>
-      <c r="B17" t="s">
-        <v>111</v>
-      </c>
-      <c r="C17" t="s">
-        <v>112</v>
-      </c>
-      <c r="D17" t="s">
-        <v>911</v>
-      </c>
-      <c r="E17" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>899</v>
-      </c>
-      <c r="B18" t="s">
-        <v>116</v>
-      </c>
-      <c r="C18" t="s">
-        <v>117</v>
-      </c>
-      <c r="D18" t="s">
-        <v>912</v>
-      </c>
-      <c r="E18" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>900</v>
-      </c>
-      <c r="B19" t="s">
-        <v>123</v>
-      </c>
-      <c r="C19" t="s">
-        <v>124</v>
-      </c>
-      <c r="D19" t="s">
-        <v>587</v>
-      </c>
-      <c r="E19" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>901</v>
-      </c>
-      <c r="B20" t="s">
-        <v>130</v>
-      </c>
-      <c r="C20" t="s">
-        <v>131</v>
-      </c>
-      <c r="D20" t="s">
-        <v>533</v>
-      </c>
-      <c r="E20" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>902</v>
-      </c>
-      <c r="B21" t="s">
-        <v>136</v>
-      </c>
-      <c r="C21" t="s">
-        <v>137</v>
-      </c>
-      <c r="D21" t="s">
-        <v>913</v>
-      </c>
-      <c r="E21" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>903</v>
-      </c>
-      <c r="B22" t="s">
-        <v>141</v>
-      </c>
-      <c r="C22" t="s">
-        <v>142</v>
-      </c>
-      <c r="D22" t="s">
-        <v>142</v>
-      </c>
-      <c r="E22" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>904</v>
-      </c>
-      <c r="B23" t="s">
-        <v>148</v>
-      </c>
-      <c r="C23" t="s">
-        <v>149</v>
-      </c>
-      <c r="D23" t="s">
-        <v>149</v>
-      </c>
-      <c r="E23" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
-        <v>905</v>
-      </c>
-      <c r="B24" t="s">
-        <v>155</v>
-      </c>
-      <c r="C24" t="s">
-        <v>156</v>
-      </c>
-      <c r="D24" t="s">
-        <v>156</v>
-      </c>
-      <c r="E24" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
-        <v>906</v>
-      </c>
-      <c r="B25" t="s">
-        <v>162</v>
-      </c>
-      <c r="C25" t="s">
-        <v>163</v>
-      </c>
-      <c r="D25" t="s">
-        <v>163</v>
-      </c>
-      <c r="E25" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
-        <v>907</v>
-      </c>
-      <c r="B26" t="s">
-        <v>168</v>
-      </c>
-      <c r="C26" t="s">
-        <v>169</v>
-      </c>
-      <c r="D26" t="s">
-        <v>169</v>
-      </c>
-      <c r="E26" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
-        <v>908</v>
-      </c>
-      <c r="B27" t="s">
-        <v>175</v>
-      </c>
-      <c r="C27" t="s">
-        <v>176</v>
-      </c>
-      <c r="D27" t="s">
-        <v>176</v>
-      </c>
-      <c r="E27" t="s">
-        <v>176</v>
+      <c r="D27" s="15" t="s">
+        <v>184</v>
+      </c>
+      <c r="E27" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="F27" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="G27" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="H27" s="15" t="s">
+        <v>186</v>
+      </c>
+      <c r="I27" s="15" t="s">
+        <v>187</v>
+      </c>
+      <c r="J27" s="15" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="57" x14ac:dyDescent="0.2">
+      <c r="A28" s="16" t="s">
+        <v>189</v>
+      </c>
+      <c r="B28" s="16" t="s">
+        <v>190</v>
+      </c>
+      <c r="C28" s="16" t="s">
+        <v>191</v>
+      </c>
+      <c r="D28" s="16" t="s">
+        <v>191</v>
+      </c>
+      <c r="E28" s="16" t="s">
+        <v>191</v>
+      </c>
+      <c r="F28" s="16" t="s">
+        <v>191</v>
+      </c>
+      <c r="G28" s="16" t="s">
+        <v>191</v>
+      </c>
+      <c r="H28" s="16" t="s">
+        <v>191</v>
+      </c>
+      <c r="I28" s="16" t="s">
+        <v>191</v>
+      </c>
+      <c r="J28" s="16" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="38" x14ac:dyDescent="0.2">
+      <c r="A29" s="16" t="s">
+        <v>193</v>
+      </c>
+      <c r="B29" s="16" t="s">
+        <v>194</v>
+      </c>
+      <c r="C29" s="16" t="s">
+        <v>191</v>
+      </c>
+      <c r="D29" s="16" t="s">
+        <v>191</v>
+      </c>
+      <c r="E29" s="16" t="s">
+        <v>191</v>
+      </c>
+      <c r="F29" s="16" t="s">
+        <v>191</v>
+      </c>
+      <c r="G29" s="16" t="s">
+        <v>191</v>
+      </c>
+      <c r="H29" s="16" t="s">
+        <v>191</v>
+      </c>
+      <c r="I29" s="16" t="s">
+        <v>191</v>
+      </c>
+      <c r="J29" s="16" t="s">
+        <v>195</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <autoFilter ref="A1:J29" xr:uid="{00000000-0001-0000-0300-000000000000}"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="8" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <headerFooter>
+    <oddFooter>&amp;L&amp;"Aptos"&amp;10 &amp;K000000_x000D_# Public</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -6227,545 +6707,558 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G26"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.5703125" defaultRowHeight="32.5" customHeight="1" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1908BFEF-047E-5F45-B558-E6F9CE558EF2}">
+  <dimension ref="A1:F27"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="18" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.5703125" style="13" customWidth="1"/>
-    <col min="2" max="2" width="63.85546875" style="10" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="72" style="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="36.42578125" style="13" customWidth="1"/>
-    <col min="5" max="5" width="25.85546875" style="13" customWidth="1"/>
-    <col min="6" max="6" width="69" style="10" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="43.42578125" style="12" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="14.5703125" style="10" customWidth="1"/>
-    <col min="10" max="16384" width="14.5703125" style="10"/>
+    <col min="1" max="2" width="13" customWidth="1"/>
+    <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="46.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="67.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="38" t="s">
-        <v>274</v>
-      </c>
-      <c r="B1" s="45" t="s">
-        <v>275</v>
-      </c>
-      <c r="C1" s="45" t="s">
-        <v>276</v>
-      </c>
-      <c r="D1" s="38" t="s">
-        <v>277</v>
-      </c>
-      <c r="E1" s="38" t="s">
-        <v>234</v>
-      </c>
-      <c r="F1" s="45" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="46">
+    <row r="1" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A1" s="14" t="s">
+        <v>881</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="47" t="s">
+      <c r="D1" s="14" t="s">
+        <v>630</v>
+      </c>
+      <c r="E1" s="14" t="s">
+        <v>914</v>
+      </c>
+      <c r="F1" s="14" t="s">
+        <v>882</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A2" s="15" t="s">
+        <v>883</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" s="15" t="s">
         <v>279</v>
       </c>
-      <c r="C2" s="47" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" s="46" t="s">
-        <v>280</v>
-      </c>
-      <c r="E2" s="48" t="s">
-        <v>281</v>
-      </c>
-      <c r="F2" s="47" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="46">
-        <v>2</v>
-      </c>
-      <c r="B3" s="47" t="s">
+    </row>
+    <row r="3" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A3" s="15" t="s">
+        <v>884</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" s="15" t="s">
         <v>279</v>
       </c>
-      <c r="C3" s="47" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" s="46" t="s">
-        <v>280</v>
-      </c>
-      <c r="E3" s="49" t="s">
-        <v>243</v>
-      </c>
-      <c r="F3" s="47" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="46">
-        <v>3</v>
-      </c>
-      <c r="B4" s="47" t="s">
+    </row>
+    <row r="4" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A4" s="15" t="s">
+        <v>885</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" s="15" t="s">
+        <v>250</v>
+      </c>
+      <c r="F4" s="15" t="s">
         <v>279</v>
       </c>
-      <c r="C4" s="47" t="s">
-        <v>29</v>
-      </c>
-      <c r="D4" s="46" t="s">
-        <v>284</v>
-      </c>
-      <c r="E4" s="49" t="s">
-        <v>243</v>
-      </c>
-      <c r="F4" s="47" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="46">
-        <v>4</v>
-      </c>
-      <c r="B5" s="47" t="s">
+    </row>
+    <row r="5" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A5" s="15" t="s">
+        <v>886</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="F5" s="15" t="s">
         <v>279</v>
       </c>
-      <c r="C5" s="47" t="s">
-        <v>36</v>
-      </c>
-      <c r="D5" s="46"/>
-      <c r="E5" s="49" t="s">
-        <v>243</v>
-      </c>
-      <c r="F5" s="47" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="46">
-        <v>5</v>
-      </c>
-      <c r="B6" s="47" t="s">
+    </row>
+    <row r="6" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A6" s="15" t="s">
+        <v>887</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="F6" s="15" t="s">
         <v>279</v>
       </c>
-      <c r="C6" s="47" t="s">
-        <v>44</v>
-      </c>
-      <c r="D6" s="46" t="s">
-        <v>280</v>
-      </c>
-      <c r="E6" s="49" t="s">
-        <v>243</v>
-      </c>
-      <c r="F6" s="47" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="46">
-        <v>6</v>
-      </c>
-      <c r="B7" s="47" t="s">
+    </row>
+    <row r="7" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A7" s="15" t="s">
+        <v>888</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="F7" s="15" t="s">
         <v>279</v>
       </c>
-      <c r="C7" s="47" t="s">
-        <v>50</v>
-      </c>
-      <c r="D7" s="46" t="s">
-        <v>284</v>
-      </c>
-      <c r="E7" s="49" t="s">
-        <v>243</v>
-      </c>
-      <c r="F7" s="47" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="46">
-        <v>7</v>
-      </c>
-      <c r="B8" s="47" t="s">
+    </row>
+    <row r="8" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A8" s="15" t="s">
+        <v>889</v>
+      </c>
+      <c r="B8" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="F8" s="15" t="s">
         <v>279</v>
       </c>
-      <c r="C8" s="47" t="s">
-        <v>57</v>
-      </c>
-      <c r="D8" s="46" t="s">
-        <v>284</v>
-      </c>
-      <c r="E8" s="49" t="s">
-        <v>243</v>
-      </c>
-      <c r="F8" s="47" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="46">
-        <v>8</v>
-      </c>
-      <c r="B9" s="47" t="s">
+    </row>
+    <row r="9" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A9" s="15" t="s">
+        <v>890</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="F9" s="15" t="s">
         <v>279</v>
       </c>
-      <c r="C9" s="47" t="s">
-        <v>63</v>
-      </c>
-      <c r="D9" s="46" t="s">
-        <v>290</v>
-      </c>
-      <c r="E9" s="48" t="s">
-        <v>281</v>
-      </c>
-      <c r="F9" s="47" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="46">
-        <v>9</v>
-      </c>
-      <c r="B10" s="47" t="s">
+    </row>
+    <row r="10" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A10" s="15" t="s">
+        <v>891</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="F10" s="15" t="s">
         <v>279</v>
       </c>
-      <c r="C10" s="47" t="s">
-        <v>70</v>
-      </c>
-      <c r="D10" s="46" t="s">
-        <v>292</v>
-      </c>
-      <c r="E10" s="49" t="s">
-        <v>243</v>
-      </c>
-      <c r="F10" s="47" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="46">
-        <v>10</v>
-      </c>
-      <c r="B11" s="47" t="s">
+    </row>
+    <row r="11" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A11" s="15" t="s">
+        <v>892</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="F11" s="15" t="s">
         <v>294</v>
       </c>
-      <c r="C11" s="47" t="s">
-        <v>77</v>
-      </c>
-      <c r="D11" s="46" t="s">
-        <v>280</v>
-      </c>
-      <c r="E11" s="49" t="s">
-        <v>243</v>
-      </c>
-      <c r="F11" s="47" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="46">
+    </row>
+    <row r="12" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A12" s="15" t="s">
+        <v>893</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="C12" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="47" t="s">
+      <c r="D12" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="E12" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="F12" s="15" t="s">
         <v>294</v>
       </c>
-      <c r="C12" s="47" t="s">
-        <v>84</v>
-      </c>
-      <c r="D12" s="46" t="s">
-        <v>284</v>
-      </c>
-      <c r="E12" s="49" t="s">
-        <v>243</v>
-      </c>
-      <c r="F12" s="47" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="46">
-        <v>12</v>
-      </c>
-      <c r="B13" s="47" t="s">
+    </row>
+    <row r="13" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A13" s="15" t="s">
+        <v>894</v>
+      </c>
+      <c r="B13" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="E13" s="15" t="s">
+        <v>271</v>
+      </c>
+      <c r="F13" s="15" t="s">
         <v>294</v>
       </c>
-      <c r="C13" s="47" t="s">
-        <v>91</v>
-      </c>
-      <c r="D13" s="46" t="s">
-        <v>280</v>
-      </c>
-      <c r="E13" s="49" t="s">
-        <v>243</v>
-      </c>
-      <c r="F13" s="47" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="46">
-        <v>13</v>
-      </c>
-      <c r="B14" s="47" t="s">
+    </row>
+    <row r="14" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A14" s="15" t="s">
+        <v>895</v>
+      </c>
+      <c r="B14" s="15" t="s">
+        <v>97</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="E14" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="F14" s="15" t="s">
         <v>294</v>
       </c>
-      <c r="C14" s="47" t="s">
-        <v>98</v>
-      </c>
-      <c r="D14" s="46" t="s">
-        <v>280</v>
-      </c>
-      <c r="E14" s="49" t="s">
-        <v>243</v>
-      </c>
-      <c r="F14" s="47" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="46">
-        <v>14</v>
-      </c>
-      <c r="B15" s="47" t="s">
+    </row>
+    <row r="15" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A15" s="15" t="s">
+        <v>896</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="E15" s="15" t="s">
+        <v>909</v>
+      </c>
+      <c r="F15" s="15" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A16" s="15" t="s">
+        <v>897</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="C16" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="E16" s="15" t="s">
+        <v>910</v>
+      </c>
+      <c r="F16" s="15" t="s">
         <v>299</v>
       </c>
-      <c r="C15" s="47" t="s">
-        <v>105</v>
-      </c>
-      <c r="D15" s="46" t="s">
-        <v>290</v>
-      </c>
-      <c r="E15" s="50" t="s">
-        <v>246</v>
-      </c>
-      <c r="F15" s="47" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="46">
-        <v>15</v>
-      </c>
-      <c r="B16" s="47" t="s">
+    </row>
+    <row r="17" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A17" s="15" t="s">
+        <v>898</v>
+      </c>
+      <c r="B17" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C17" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="E17" s="15" t="s">
+        <v>911</v>
+      </c>
+      <c r="F17" s="15" t="s">
         <v>299</v>
       </c>
-      <c r="C16" s="47" t="s">
-        <v>112</v>
-      </c>
-      <c r="D16" s="46" t="s">
-        <v>290</v>
-      </c>
-      <c r="E16" s="50" t="s">
-        <v>246</v>
-      </c>
-      <c r="F16" s="47" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="46">
-        <v>16</v>
-      </c>
-      <c r="B17" s="47" t="s">
+    </row>
+    <row r="18" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A18" s="15" t="s">
+        <v>899</v>
+      </c>
+      <c r="B18" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="C18" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="E18" s="15" t="s">
+        <v>912</v>
+      </c>
+      <c r="F18" s="15" t="s">
         <v>299</v>
       </c>
-      <c r="C17" s="47" t="s">
-        <v>117</v>
-      </c>
-      <c r="D17" s="46" t="s">
-        <v>290</v>
-      </c>
-      <c r="E17" s="49" t="s">
-        <v>243</v>
-      </c>
-      <c r="F17" s="47" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="46">
-        <v>17</v>
-      </c>
-      <c r="B18" s="47" t="s">
+    </row>
+    <row r="19" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A19" s="15" t="s">
+        <v>900</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="C19" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="E19" s="15" t="s">
+        <v>587</v>
+      </c>
+      <c r="F19" s="15" t="s">
         <v>299</v>
       </c>
-      <c r="C18" s="47" t="s">
-        <v>124</v>
-      </c>
-      <c r="D18" s="46" t="s">
-        <v>302</v>
-      </c>
-      <c r="E18" s="48" t="s">
-        <v>281</v>
-      </c>
-      <c r="F18" s="47" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="46">
-        <v>18</v>
-      </c>
-      <c r="B19" s="47" t="s">
+    </row>
+    <row r="20" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A20" s="15" t="s">
+        <v>901</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="C20" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="E20" s="15" t="s">
+        <v>533</v>
+      </c>
+      <c r="F20" s="15" t="s">
         <v>304</v>
       </c>
-      <c r="C19" s="47" t="s">
-        <v>131</v>
-      </c>
-      <c r="D19" s="46" t="s">
-        <v>290</v>
-      </c>
-      <c r="E19" s="49" t="s">
-        <v>243</v>
-      </c>
-      <c r="F19" s="47" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="46">
-        <v>19</v>
-      </c>
-      <c r="B20" s="47" t="s">
+    </row>
+    <row r="21" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A21" s="15" t="s">
+        <v>902</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="C21" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="E21" s="15" t="s">
+        <v>913</v>
+      </c>
+      <c r="F21" s="15" t="s">
         <v>304</v>
       </c>
-      <c r="C20" s="47" t="s">
-        <v>137</v>
-      </c>
-      <c r="D20" s="46" t="s">
-        <v>290</v>
-      </c>
-      <c r="E20" s="49" t="s">
-        <v>243</v>
-      </c>
-      <c r="F20" s="47" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="46">
-        <v>20</v>
-      </c>
-      <c r="B21" s="47" t="s">
+    </row>
+    <row r="22" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A22" s="15" t="s">
+        <v>903</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="C22" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D22" s="15" t="s">
+        <v>142</v>
+      </c>
+      <c r="E22" s="15" t="s">
+        <v>142</v>
+      </c>
+      <c r="F22" s="15" t="s">
         <v>307</v>
       </c>
-      <c r="C21" s="47" t="s">
-        <v>142</v>
-      </c>
-      <c r="D21" s="46" t="s">
-        <v>290</v>
-      </c>
-      <c r="E21" s="50" t="s">
-        <v>246</v>
-      </c>
-      <c r="F21" s="47" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="46">
-        <v>21</v>
-      </c>
-      <c r="B22" s="47" t="s">
+    </row>
+    <row r="23" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A23" s="15" t="s">
+        <v>904</v>
+      </c>
+      <c r="B23" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="C23" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="E23" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="F23" s="15" t="s">
         <v>307</v>
       </c>
-      <c r="C22" s="47" t="s">
-        <v>149</v>
-      </c>
-      <c r="D22" s="46" t="s">
-        <v>290</v>
-      </c>
-      <c r="E22" s="50" t="s">
-        <v>246</v>
-      </c>
-      <c r="F22" s="47" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="46">
-        <v>22</v>
-      </c>
-      <c r="B23" s="47" t="s">
+    </row>
+    <row r="24" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A24" s="15" t="s">
+        <v>905</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="C24" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24" s="15" t="s">
+        <v>156</v>
+      </c>
+      <c r="E24" s="15" t="s">
+        <v>156</v>
+      </c>
+      <c r="F24" s="15" t="s">
         <v>310</v>
       </c>
-      <c r="C23" s="47" t="s">
-        <v>156</v>
-      </c>
-      <c r="D23" s="46" t="s">
-        <v>311</v>
-      </c>
-      <c r="E23" s="48" t="s">
-        <v>281</v>
-      </c>
-      <c r="F23" s="47" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="46">
-        <v>23</v>
-      </c>
-      <c r="B24" s="47" t="s">
+    </row>
+    <row r="25" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A25" s="15" t="s">
+        <v>906</v>
+      </c>
+      <c r="B25" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="C25" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="E25" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="F25" s="15" t="s">
         <v>310</v>
       </c>
-      <c r="C24" s="47" t="s">
-        <v>163</v>
-      </c>
-      <c r="D24" s="46" t="s">
-        <v>311</v>
-      </c>
-      <c r="E24" s="48" t="s">
-        <v>281</v>
-      </c>
-      <c r="F24" s="47" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="46">
-        <v>24</v>
-      </c>
-      <c r="B25" s="47" t="s">
+    </row>
+    <row r="26" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A26" s="15" t="s">
+        <v>907</v>
+      </c>
+      <c r="B26" s="15" t="s">
+        <v>168</v>
+      </c>
+      <c r="C26" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D26" s="15" t="s">
+        <v>169</v>
+      </c>
+      <c r="E26" s="15" t="s">
+        <v>169</v>
+      </c>
+      <c r="F26" s="15" t="s">
         <v>172</v>
       </c>
-      <c r="C25" s="47" t="s">
-        <v>169</v>
-      </c>
-      <c r="D25" s="46" t="s">
-        <v>314</v>
-      </c>
-      <c r="E25" s="50" t="s">
-        <v>246</v>
-      </c>
-      <c r="F25" s="47" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="46">
-        <v>25</v>
-      </c>
-      <c r="B26" s="47" t="s">
+    </row>
+    <row r="27" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A27" s="15" t="s">
+        <v>908</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>175</v>
+      </c>
+      <c r="C27" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D27" s="15" t="s">
         <v>176</v>
       </c>
-      <c r="C26" s="47" t="s">
+      <c r="E27" s="15" t="s">
         <v>176</v>
       </c>
-      <c r="D26" s="46" t="s">
-        <v>290</v>
-      </c>
-      <c r="E26" s="46" t="s">
-        <v>316</v>
-      </c>
-      <c r="F26" s="47" t="s">
-        <v>317</v>
+      <c r="F27" s="15" t="s">
+        <v>176</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1" xr:uid="{00000000-0009-0000-0000-000002000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F27">
-      <sortCondition ref="A1:A27"/>
-    </sortState>
-  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
@@ -7179,20 +7672,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="59" t="s">
         <v>196</v>
       </c>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="61" t="s">
+      <c r="A2" s="60" t="s">
         <v>197</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
+      <c r="B2" s="61"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="25"/>
@@ -7393,959 +7886,547 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:J29"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.85546875" defaultRowHeight="18" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:G26"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.5703125" defaultRowHeight="32.5" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="15.5703125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="34.5703125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="29.7109375" style="3" customWidth="1"/>
-    <col min="5" max="5" width="27" style="3" customWidth="1"/>
-    <col min="6" max="6" width="24.28515625" style="3" customWidth="1"/>
-    <col min="7" max="7" width="32.42578125" style="3" customWidth="1"/>
-    <col min="8" max="8" width="24.28515625" style="3" customWidth="1"/>
-    <col min="9" max="9" width="21.5703125" style="3" customWidth="1"/>
-    <col min="10" max="10" width="81" style="3" customWidth="1"/>
-    <col min="11" max="13" width="11.85546875" style="1" customWidth="1"/>
-    <col min="14" max="16384" width="11.85546875" style="1"/>
+    <col min="1" max="1" width="14.5703125" style="13" customWidth="1"/>
+    <col min="2" max="2" width="63.85546875" style="10" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="72" style="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36.42578125" style="13" customWidth="1"/>
+    <col min="5" max="5" width="25.85546875" style="13" customWidth="1"/>
+    <col min="6" max="6" width="69" style="10" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="43.42578125" style="12" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="14.5703125" style="10" customWidth="1"/>
+    <col min="10" max="16384" width="14.5703125" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="37.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="14" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="14" t="s">
+    <row r="1" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="38" t="s">
+        <v>274</v>
+      </c>
+      <c r="B1" s="45" t="s">
+        <v>275</v>
+      </c>
+      <c r="C1" s="45" t="s">
+        <v>276</v>
+      </c>
+      <c r="D1" s="38" t="s">
+        <v>277</v>
+      </c>
+      <c r="E1" s="38" t="s">
+        <v>234</v>
+      </c>
+      <c r="F1" s="45" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="46">
         <v>1</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="B2" s="47" t="s">
+        <v>279</v>
+      </c>
+      <c r="C2" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="46" t="s">
+        <v>280</v>
+      </c>
+      <c r="E2" s="48" t="s">
+        <v>281</v>
+      </c>
+      <c r="F2" s="47" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="46">
         <v>2</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="B3" s="47" t="s">
+        <v>279</v>
+      </c>
+      <c r="C3" s="47" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="46" t="s">
+        <v>280</v>
+      </c>
+      <c r="E3" s="49" t="s">
+        <v>243</v>
+      </c>
+      <c r="F3" s="47" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="46">
         <v>3</v>
       </c>
-      <c r="E1" s="14" t="s">
+      <c r="B4" s="47" t="s">
+        <v>279</v>
+      </c>
+      <c r="C4" s="47" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="46" t="s">
+        <v>284</v>
+      </c>
+      <c r="E4" s="49" t="s">
+        <v>243</v>
+      </c>
+      <c r="F4" s="47" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="46">
         <v>4</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="B5" s="47" t="s">
+        <v>279</v>
+      </c>
+      <c r="C5" s="47" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="46"/>
+      <c r="E5" s="49" t="s">
+        <v>243</v>
+      </c>
+      <c r="F5" s="47" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="46">
         <v>5</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="B6" s="47" t="s">
+        <v>279</v>
+      </c>
+      <c r="C6" s="47" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="46" t="s">
+        <v>280</v>
+      </c>
+      <c r="E6" s="49" t="s">
+        <v>243</v>
+      </c>
+      <c r="F6" s="47" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="46">
         <v>6</v>
       </c>
-      <c r="H1" s="14" t="s">
+      <c r="B7" s="47" t="s">
+        <v>279</v>
+      </c>
+      <c r="C7" s="47" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" s="46" t="s">
+        <v>284</v>
+      </c>
+      <c r="E7" s="49" t="s">
+        <v>243</v>
+      </c>
+      <c r="F7" s="47" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="46">
         <v>7</v>
       </c>
-      <c r="I1" s="14" t="s">
+      <c r="B8" s="47" t="s">
+        <v>279</v>
+      </c>
+      <c r="C8" s="47" t="s">
+        <v>57</v>
+      </c>
+      <c r="D8" s="46" t="s">
+        <v>284</v>
+      </c>
+      <c r="E8" s="49" t="s">
+        <v>243</v>
+      </c>
+      <c r="F8" s="47" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="46">
         <v>8</v>
       </c>
-      <c r="J1" s="14" t="s">
+      <c r="B9" s="47" t="s">
+        <v>279</v>
+      </c>
+      <c r="C9" s="47" t="s">
+        <v>63</v>
+      </c>
+      <c r="D9" s="46" t="s">
+        <v>290</v>
+      </c>
+      <c r="E9" s="48" t="s">
+        <v>281</v>
+      </c>
+      <c r="F9" s="47" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="46">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="15" t="s">
+      <c r="B10" s="47" t="s">
+        <v>279</v>
+      </c>
+      <c r="C10" s="47" t="s">
+        <v>70</v>
+      </c>
+      <c r="D10" s="46" t="s">
+        <v>292</v>
+      </c>
+      <c r="E10" s="49" t="s">
+        <v>243</v>
+      </c>
+      <c r="F10" s="47" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="46">
         <v>10</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B11" s="47" t="s">
+        <v>294</v>
+      </c>
+      <c r="C11" s="47" t="s">
+        <v>77</v>
+      </c>
+      <c r="D11" s="46" t="s">
+        <v>280</v>
+      </c>
+      <c r="E11" s="49" t="s">
+        <v>243</v>
+      </c>
+      <c r="F11" s="47" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="46">
         <v>11</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="B12" s="47" t="s">
+        <v>294</v>
+      </c>
+      <c r="C12" s="47" t="s">
+        <v>84</v>
+      </c>
+      <c r="D12" s="46" t="s">
+        <v>284</v>
+      </c>
+      <c r="E12" s="49" t="s">
+        <v>243</v>
+      </c>
+      <c r="F12" s="47" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="46">
         <v>12</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="B13" s="47" t="s">
+        <v>294</v>
+      </c>
+      <c r="C13" s="47" t="s">
+        <v>91</v>
+      </c>
+      <c r="D13" s="46" t="s">
+        <v>280</v>
+      </c>
+      <c r="E13" s="49" t="s">
+        <v>243</v>
+      </c>
+      <c r="F13" s="47" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="46">
         <v>13</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="B14" s="47" t="s">
+        <v>294</v>
+      </c>
+      <c r="C14" s="47" t="s">
+        <v>98</v>
+      </c>
+      <c r="D14" s="46" t="s">
+        <v>280</v>
+      </c>
+      <c r="E14" s="49" t="s">
+        <v>243</v>
+      </c>
+      <c r="F14" s="47" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="46">
         <v>14</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="B15" s="47" t="s">
+        <v>299</v>
+      </c>
+      <c r="C15" s="47" t="s">
+        <v>105</v>
+      </c>
+      <c r="D15" s="46" t="s">
+        <v>290</v>
+      </c>
+      <c r="E15" s="50" t="s">
+        <v>246</v>
+      </c>
+      <c r="F15" s="47" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="46">
         <v>15</v>
       </c>
-      <c r="G2" s="15" t="s">
+      <c r="B16" s="47" t="s">
+        <v>299</v>
+      </c>
+      <c r="C16" s="47" t="s">
+        <v>112</v>
+      </c>
+      <c r="D16" s="46" t="s">
+        <v>290</v>
+      </c>
+      <c r="E16" s="50" t="s">
+        <v>246</v>
+      </c>
+      <c r="F16" s="47" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="46">
         <v>16</v>
       </c>
-      <c r="H2" s="15" t="s">
+      <c r="B17" s="47" t="s">
+        <v>299</v>
+      </c>
+      <c r="C17" s="47" t="s">
+        <v>117</v>
+      </c>
+      <c r="D17" s="46" t="s">
+        <v>290</v>
+      </c>
+      <c r="E17" s="49" t="s">
+        <v>243</v>
+      </c>
+      <c r="F17" s="47" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="46">
         <v>17</v>
       </c>
-      <c r="I2" s="15" t="s">
+      <c r="B18" s="47" t="s">
+        <v>299</v>
+      </c>
+      <c r="C18" s="47" t="s">
+        <v>124</v>
+      </c>
+      <c r="D18" s="46" t="s">
+        <v>302</v>
+      </c>
+      <c r="E18" s="48" t="s">
+        <v>281</v>
+      </c>
+      <c r="F18" s="47" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="46">
         <v>18</v>
       </c>
-      <c r="J2" s="15" t="s">
+      <c r="B19" s="47" t="s">
+        <v>304</v>
+      </c>
+      <c r="C19" s="47" t="s">
+        <v>131</v>
+      </c>
+      <c r="D19" s="46" t="s">
+        <v>290</v>
+      </c>
+      <c r="E19" s="49" t="s">
+        <v>243</v>
+      </c>
+      <c r="F19" s="47" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="46">
         <v>19</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="15" t="s">
+      <c r="B20" s="47" t="s">
+        <v>304</v>
+      </c>
+      <c r="C20" s="47" t="s">
+        <v>137</v>
+      </c>
+      <c r="D20" s="46" t="s">
+        <v>290</v>
+      </c>
+      <c r="E20" s="49" t="s">
+        <v>243</v>
+      </c>
+      <c r="F20" s="47" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="46">
         <v>20</v>
       </c>
-      <c r="B3" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="15" t="s">
+      <c r="B21" s="47" t="s">
+        <v>307</v>
+      </c>
+      <c r="C21" s="47" t="s">
+        <v>142</v>
+      </c>
+      <c r="D21" s="46" t="s">
+        <v>290</v>
+      </c>
+      <c r="E21" s="50" t="s">
+        <v>246</v>
+      </c>
+      <c r="F21" s="47" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="46">
         <v>21</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="B22" s="47" t="s">
+        <v>307</v>
+      </c>
+      <c r="C22" s="47" t="s">
+        <v>149</v>
+      </c>
+      <c r="D22" s="46" t="s">
+        <v>290</v>
+      </c>
+      <c r="E22" s="50" t="s">
+        <v>246</v>
+      </c>
+      <c r="F22" s="47" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="46">
         <v>22</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="B23" s="47" t="s">
+        <v>310</v>
+      </c>
+      <c r="C23" s="47" t="s">
+        <v>156</v>
+      </c>
+      <c r="D23" s="46" t="s">
+        <v>311</v>
+      </c>
+      <c r="E23" s="48" t="s">
+        <v>281</v>
+      </c>
+      <c r="F23" s="47" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="46">
         <v>23</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="B24" s="47" t="s">
+        <v>310</v>
+      </c>
+      <c r="C24" s="47" t="s">
+        <v>163</v>
+      </c>
+      <c r="D24" s="46" t="s">
+        <v>311</v>
+      </c>
+      <c r="E24" s="48" t="s">
+        <v>281</v>
+      </c>
+      <c r="F24" s="47" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="46">
         <v>24</v>
       </c>
-      <c r="G3" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3" s="15" t="s">
+      <c r="B25" s="47" t="s">
+        <v>172</v>
+      </c>
+      <c r="C25" s="47" t="s">
+        <v>169</v>
+      </c>
+      <c r="D25" s="46" t="s">
+        <v>314</v>
+      </c>
+      <c r="E25" s="50" t="s">
+        <v>246</v>
+      </c>
+      <c r="F25" s="47" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="46">
         <v>25</v>
       </c>
-      <c r="I3" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="J3" s="15" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B4" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="E4" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="G4" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="H4" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="I4" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="J4" s="15" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="B5" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="D5" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="E5" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="F5" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="G5" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="H5" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="I5" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="J5" s="15" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="B6" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="G6" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="H6" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="I6" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="J6" s="15" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="15" t="s">
-        <v>49</v>
-      </c>
-      <c r="B7" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="D7" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="E7" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="F7" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="G7" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="H7" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="I7" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="J7" s="15" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="B8" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="D8" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="E8" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="F8" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="G8" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="H8" s="15" t="s">
-        <v>59</v>
-      </c>
-      <c r="I8" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="J8" s="15" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="B9" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="D9" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="E9" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="F9" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="G9" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="H9" s="15" t="s">
-        <v>66</v>
-      </c>
-      <c r="I9" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="J9" s="15" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="B10" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="D10" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="E10" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="F10" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="G10" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="H10" s="15" t="s">
-        <v>73</v>
-      </c>
-      <c r="I10" s="15" t="s">
-        <v>74</v>
-      </c>
-      <c r="J10" s="15" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="64.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="B11" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C11" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="D11" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="E11" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="F11" s="15" t="s">
-        <v>79</v>
-      </c>
-      <c r="G11" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="H11" s="15" t="s">
-        <v>80</v>
-      </c>
-      <c r="I11" s="15" t="s">
-        <v>81</v>
-      </c>
-      <c r="J11" s="15" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="64.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="15" t="s">
-        <v>83</v>
-      </c>
-      <c r="B12" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C12" s="15" t="s">
-        <v>84</v>
-      </c>
-      <c r="D12" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="E12" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="F12" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="G12" s="15" t="s">
-        <v>84</v>
-      </c>
-      <c r="H12" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="I12" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="J12" s="15" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="86.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="B13" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C13" s="15" t="s">
-        <v>91</v>
-      </c>
-      <c r="D13" s="15" t="s">
-        <v>92</v>
-      </c>
-      <c r="E13" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="F13" s="15" t="s">
-        <v>93</v>
-      </c>
-      <c r="G13" s="15" t="s">
-        <v>91</v>
-      </c>
-      <c r="H13" s="15" t="s">
-        <v>94</v>
-      </c>
-      <c r="I13" s="15" t="s">
-        <v>95</v>
-      </c>
-      <c r="J13" s="15" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="64.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="15" t="s">
-        <v>97</v>
-      </c>
-      <c r="B14" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C14" s="15" t="s">
-        <v>98</v>
-      </c>
-      <c r="D14" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="E14" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="F14" s="15" t="s">
-        <v>100</v>
-      </c>
-      <c r="G14" s="15" t="s">
-        <v>98</v>
-      </c>
-      <c r="H14" s="15" t="s">
-        <v>101</v>
-      </c>
-      <c r="I14" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="J14" s="15" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="86.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="15" t="s">
-        <v>104</v>
-      </c>
-      <c r="B15" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C15" s="15" t="s">
-        <v>105</v>
-      </c>
-      <c r="D15" s="15" t="s">
-        <v>106</v>
-      </c>
-      <c r="E15" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="F15" s="15" t="s">
-        <v>107</v>
-      </c>
-      <c r="G15" s="15" t="s">
-        <v>105</v>
-      </c>
-      <c r="H15" s="15" t="s">
-        <v>108</v>
-      </c>
-      <c r="I15" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="J15" s="15" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="86.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="15" t="s">
-        <v>111</v>
-      </c>
-      <c r="B16" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C16" s="15" t="s">
-        <v>112</v>
-      </c>
-      <c r="D16" s="15" t="s">
-        <v>106</v>
-      </c>
-      <c r="E16" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="F16" s="15" t="s">
-        <v>113</v>
-      </c>
-      <c r="G16" s="15" t="s">
-        <v>112</v>
-      </c>
-      <c r="H16" s="15" t="s">
-        <v>108</v>
-      </c>
-      <c r="I16" s="15" t="s">
-        <v>114</v>
-      </c>
-      <c r="J16" s="15" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="86.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="15" t="s">
-        <v>116</v>
-      </c>
-      <c r="B17" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C17" s="15" t="s">
-        <v>117</v>
-      </c>
-      <c r="D17" s="15" t="s">
-        <v>106</v>
-      </c>
-      <c r="E17" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="F17" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="G17" s="15" t="s">
-        <v>119</v>
-      </c>
-      <c r="H17" s="15" t="s">
-        <v>120</v>
-      </c>
-      <c r="I17" s="15" t="s">
-        <v>121</v>
-      </c>
-      <c r="J17" s="15" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="64.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="15" t="s">
-        <v>123</v>
-      </c>
-      <c r="B18" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C18" s="15" t="s">
-        <v>124</v>
-      </c>
-      <c r="D18" s="15" t="s">
-        <v>106</v>
-      </c>
-      <c r="E18" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="F18" s="15" t="s">
-        <v>125</v>
-      </c>
-      <c r="G18" s="15" t="s">
-        <v>126</v>
-      </c>
-      <c r="H18" s="15" t="s">
-        <v>127</v>
-      </c>
-      <c r="I18" s="15" t="s">
-        <v>128</v>
-      </c>
-      <c r="J18" s="15" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="86.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="15" t="s">
-        <v>130</v>
-      </c>
-      <c r="B19" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C19" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="D19" s="15" t="s">
-        <v>106</v>
-      </c>
-      <c r="E19" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="F19" s="15" t="s">
-        <v>132</v>
-      </c>
-      <c r="G19" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="H19" s="15" t="s">
-        <v>133</v>
-      </c>
-      <c r="I19" s="15" t="s">
-        <v>134</v>
-      </c>
-      <c r="J19" s="15" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="86.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="B20" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C20" s="15" t="s">
-        <v>137</v>
-      </c>
-      <c r="D20" s="15" t="s">
-        <v>106</v>
-      </c>
-      <c r="E20" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="F20" s="15" t="s">
-        <v>138</v>
-      </c>
-      <c r="G20" s="15" t="s">
-        <v>137</v>
-      </c>
-      <c r="H20" s="15" t="s">
-        <v>139</v>
-      </c>
-      <c r="I20" s="15" t="s">
-        <v>140</v>
-      </c>
-      <c r="J20" s="15" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="64.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="15" t="s">
-        <v>141</v>
-      </c>
-      <c r="B21" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C21" s="15" t="s">
-        <v>142</v>
-      </c>
-      <c r="D21" s="15" t="s">
-        <v>143</v>
-      </c>
-      <c r="E21" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="F21" s="15" t="s">
-        <v>144</v>
-      </c>
-      <c r="G21" s="15" t="s">
-        <v>142</v>
-      </c>
-      <c r="H21" s="15" t="s">
-        <v>145</v>
-      </c>
-      <c r="I21" s="15" t="s">
-        <v>146</v>
-      </c>
-      <c r="J21" s="15" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="64.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="15" t="s">
-        <v>148</v>
-      </c>
-      <c r="B22" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C22" s="15" t="s">
-        <v>149</v>
-      </c>
-      <c r="D22" s="15" t="s">
-        <v>150</v>
-      </c>
-      <c r="E22" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="F22" s="15" t="s">
-        <v>151</v>
-      </c>
-      <c r="G22" s="15" t="s">
-        <v>149</v>
-      </c>
-      <c r="H22" s="15" t="s">
-        <v>152</v>
-      </c>
-      <c r="I22" s="15" t="s">
-        <v>153</v>
-      </c>
-      <c r="J22" s="15" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="86.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="15" t="s">
-        <v>155</v>
-      </c>
-      <c r="B23" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C23" s="15" t="s">
-        <v>156</v>
-      </c>
-      <c r="D23" s="15" t="s">
-        <v>157</v>
-      </c>
-      <c r="E23" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="F23" s="15" t="s">
-        <v>158</v>
-      </c>
-      <c r="G23" s="15" t="s">
-        <v>156</v>
-      </c>
-      <c r="H23" s="15" t="s">
-        <v>159</v>
-      </c>
-      <c r="I23" s="15" t="s">
-        <v>160</v>
-      </c>
-      <c r="J23" s="15" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="86.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="15" t="s">
-        <v>162</v>
-      </c>
-      <c r="B24" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C24" s="15" t="s">
-        <v>163</v>
-      </c>
-      <c r="D24" s="15" t="s">
-        <v>157</v>
-      </c>
-      <c r="E24" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="F24" s="15" t="s">
-        <v>164</v>
-      </c>
-      <c r="G24" s="15" t="s">
-        <v>165</v>
-      </c>
-      <c r="H24" s="15" t="s">
-        <v>166</v>
-      </c>
-      <c r="I24" s="15" t="s">
-        <v>167</v>
-      </c>
-      <c r="J24" s="15" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" ht="86.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="15" t="s">
-        <v>168</v>
-      </c>
-      <c r="B25" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C25" s="15" t="s">
-        <v>169</v>
-      </c>
-      <c r="D25" s="15" t="s">
-        <v>170</v>
-      </c>
-      <c r="E25" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="F25" s="15" t="s">
-        <v>171</v>
-      </c>
-      <c r="G25" s="15" t="s">
-        <v>169</v>
-      </c>
-      <c r="H25" s="15" t="s">
-        <v>172</v>
-      </c>
-      <c r="I25" s="15" t="s">
-        <v>173</v>
-      </c>
-      <c r="J25" s="15" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="15" t="s">
-        <v>175</v>
-      </c>
-      <c r="B26" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C26" s="15" t="s">
+      <c r="B26" s="47" t="s">
         <v>176</v>
       </c>
-      <c r="D26" s="15" t="s">
-        <v>177</v>
-      </c>
-      <c r="E26" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="F26" s="15" t="s">
-        <v>178</v>
-      </c>
-      <c r="G26" s="15" t="s">
+      <c r="C26" s="47" t="s">
         <v>176</v>
       </c>
-      <c r="H26" s="15" t="s">
-        <v>179</v>
-      </c>
-      <c r="I26" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="J26" s="15" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" ht="86.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="15" t="s">
-        <v>182</v>
-      </c>
-      <c r="B27" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C27" s="15" t="s">
-        <v>183</v>
-      </c>
-      <c r="D27" s="15" t="s">
-        <v>184</v>
-      </c>
-      <c r="E27" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="F27" s="15" t="s">
-        <v>185</v>
-      </c>
-      <c r="G27" s="15" t="s">
-        <v>183</v>
-      </c>
-      <c r="H27" s="15" t="s">
-        <v>186</v>
-      </c>
-      <c r="I27" s="15" t="s">
-        <v>187</v>
-      </c>
-      <c r="J27" s="15" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" ht="64.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="16" t="s">
-        <v>189</v>
-      </c>
-      <c r="B28" s="16" t="s">
-        <v>190</v>
-      </c>
-      <c r="C28" s="16" t="s">
-        <v>191</v>
-      </c>
-      <c r="D28" s="16" t="s">
-        <v>191</v>
-      </c>
-      <c r="E28" s="16" t="s">
-        <v>191</v>
-      </c>
-      <c r="F28" s="16" t="s">
-        <v>191</v>
-      </c>
-      <c r="G28" s="16" t="s">
-        <v>191</v>
-      </c>
-      <c r="H28" s="16" t="s">
-        <v>191</v>
-      </c>
-      <c r="I28" s="16" t="s">
-        <v>191</v>
-      </c>
-      <c r="J28" s="16" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="16" t="s">
-        <v>193</v>
-      </c>
-      <c r="B29" s="16" t="s">
-        <v>194</v>
-      </c>
-      <c r="C29" s="16" t="s">
-        <v>191</v>
-      </c>
-      <c r="D29" s="16" t="s">
-        <v>191</v>
-      </c>
-      <c r="E29" s="16" t="s">
-        <v>191</v>
-      </c>
-      <c r="F29" s="16" t="s">
-        <v>191</v>
-      </c>
-      <c r="G29" s="16" t="s">
-        <v>191</v>
-      </c>
-      <c r="H29" s="16" t="s">
-        <v>191</v>
-      </c>
-      <c r="I29" s="16" t="s">
-        <v>191</v>
-      </c>
-      <c r="J29" s="16" t="s">
-        <v>195</v>
+      <c r="D26" s="46" t="s">
+        <v>290</v>
+      </c>
+      <c r="E26" s="46" t="s">
+        <v>316</v>
+      </c>
+      <c r="F26" s="47" t="s">
+        <v>317</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J29" xr:uid="{00000000-0001-0000-0300-000000000000}"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <autoFilter ref="A1:F1" xr:uid="{00000000-0009-0000-0000-000002000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F27">
+      <sortCondition ref="A1:A27"/>
+    </sortState>
+  </autoFilter>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
-  <headerFooter>
-    <oddFooter>&amp;L&amp;"Aptos"&amp;10 &amp;K000000_x000D_# Public</oddFooter>
-  </headerFooter>
 </worksheet>
 </file>
 
@@ -8995,176 +9076,176 @@
       </c>
     </row>
     <row r="2" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="57" t="s">
         <v>374</v>
       </c>
       <c r="B2" s="21" t="s">
         <v>798</v>
       </c>
-      <c r="C2" s="59" t="s">
+      <c r="C2" s="58" t="s">
         <v>375</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="58"/>
+      <c r="A3" s="57"/>
       <c r="B3" s="21" t="s">
         <v>799</v>
       </c>
-      <c r="C3" s="59"/>
+      <c r="C3" s="58"/>
     </row>
     <row r="4" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="58"/>
+      <c r="A4" s="57"/>
       <c r="B4" s="21" t="s">
         <v>354</v>
       </c>
-      <c r="C4" s="59"/>
+      <c r="C4" s="58"/>
     </row>
     <row r="5" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="58" t="s">
+      <c r="A5" s="57" t="s">
         <v>376</v>
       </c>
       <c r="B5" s="21" t="s">
         <v>581</v>
       </c>
-      <c r="C5" s="59" t="s">
+      <c r="C5" s="58" t="s">
         <v>377</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="58"/>
+      <c r="A6" s="57"/>
       <c r="B6" s="21" t="s">
         <v>587</v>
       </c>
-      <c r="C6" s="59"/>
+      <c r="C6" s="58"/>
     </row>
     <row r="7" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="58"/>
+      <c r="A7" s="57"/>
       <c r="B7" s="21" t="s">
         <v>582</v>
       </c>
-      <c r="C7" s="59"/>
+      <c r="C7" s="58"/>
     </row>
     <row r="8" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="58" t="s">
+      <c r="A8" s="57" t="s">
         <v>378</v>
       </c>
       <c r="B8" s="21" t="s">
         <v>519</v>
       </c>
-      <c r="C8" s="59" t="s">
+      <c r="C8" s="58" t="s">
         <v>379</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="58"/>
+      <c r="A9" s="57"/>
       <c r="B9" s="21" t="s">
         <v>521</v>
       </c>
-      <c r="C9" s="59"/>
+      <c r="C9" s="58"/>
     </row>
     <row r="10" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="58" t="s">
+      <c r="A10" s="57" t="s">
         <v>380</v>
       </c>
       <c r="B10" s="21" t="s">
         <v>448</v>
       </c>
-      <c r="C10" s="59" t="s">
+      <c r="C10" s="58" t="s">
         <v>381</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="58"/>
+      <c r="A11" s="57"/>
       <c r="B11" s="21" t="s">
         <v>800</v>
       </c>
-      <c r="C11" s="59"/>
+      <c r="C11" s="58"/>
     </row>
     <row r="12" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="58"/>
+      <c r="A12" s="57"/>
       <c r="B12" s="21" t="s">
         <v>801</v>
       </c>
-      <c r="C12" s="59"/>
+      <c r="C12" s="58"/>
     </row>
     <row r="13" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="58" t="s">
+      <c r="A13" s="57" t="s">
         <v>382</v>
       </c>
       <c r="B13" s="21" t="s">
         <v>802</v>
       </c>
-      <c r="C13" s="59" t="s">
+      <c r="C13" s="58" t="s">
         <v>383</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="58"/>
+      <c r="A14" s="57"/>
       <c r="B14" s="21">
         <v>97433001001</v>
       </c>
-      <c r="C14" s="59"/>
+      <c r="C14" s="58"/>
     </row>
     <row r="15" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="58" t="s">
+      <c r="A15" s="57" t="s">
         <v>384</v>
       </c>
       <c r="B15" s="21" t="s">
         <v>803</v>
       </c>
-      <c r="C15" s="59" t="s">
+      <c r="C15" s="58" t="s">
         <v>385</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="58"/>
+      <c r="A16" s="57"/>
       <c r="B16" s="21" t="s">
         <v>804</v>
       </c>
-      <c r="C16" s="59"/>
+      <c r="C16" s="58"/>
     </row>
     <row r="17" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="58" t="s">
+      <c r="A17" s="57" t="s">
         <v>386</v>
       </c>
       <c r="B17" s="21" t="s">
         <v>805</v>
       </c>
-      <c r="C17" s="59" t="s">
+      <c r="C17" s="58" t="s">
         <v>387</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="58"/>
+      <c r="A18" s="57"/>
       <c r="B18" s="21" t="s">
         <v>806</v>
       </c>
-      <c r="C18" s="59"/>
+      <c r="C18" s="58"/>
     </row>
     <row r="19" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="58"/>
+      <c r="A19" s="57"/>
       <c r="B19" s="21" t="s">
         <v>807</v>
       </c>
-      <c r="C19" s="59"/>
+      <c r="C19" s="58"/>
     </row>
     <row r="20" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="58" t="s">
+      <c r="A20" s="57" t="s">
         <v>388</v>
       </c>
       <c r="B20" s="21" t="s">
         <v>808</v>
       </c>
-      <c r="C20" s="59" t="s">
+      <c r="C20" s="58" t="s">
         <v>389</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="58"/>
+      <c r="A21" s="57"/>
       <c r="B21" s="22" t="s">
         <v>809</v>
       </c>
-      <c r="C21" s="59"/>
+      <c r="C21" s="58"/>
     </row>
   </sheetData>
   <mergeCells count="16">

</xml_diff>